<commit_message>
test: hoan thien baseline UAT va doi chieu 40 tool
</commit_message>
<xml_diff>
--- a/outputs/uat_chatbot_dnh/uat_tracking_chatbot_dnh.xlsx
+++ b/outputs/uat_chatbot_dnh/uat_tracking_chatbot_dnh.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tổng hợp" sheetId="1" r:id="R6aa32a06b59e49ba"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checklist UAT" sheetId="2" r:id="R006c493f45304957"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hướng dẫn" sheetId="3" r:id="R19a51b2288104a56"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Danh mục" sheetId="4" r:id="R0e67ea8472cc48b5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tổng hợp" sheetId="1" r:id="Rc5e90ad0833b4e88"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checklist UAT" sheetId="2" r:id="R420e7df8aad14954"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hướng dẫn" sheetId="3" r:id="Rb106ddc774d44bf2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Danh mục" sheetId="4" r:id="Rae4be034abd84af8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -509,7 +509,7 @@
         <x:color rgb="FF375623"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE2F0D9"/>
         </x:patternFill>
       </x:fill>
@@ -520,7 +520,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE4D6"/>
         </x:patternFill>
       </x:fill>
@@ -530,7 +530,7 @@
         <x:color rgb="FF9C6500"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
@@ -541,14 +541,14 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFF4CCCC"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
@@ -925,7 +925,7 @@
       </x:c>
       <x:c r="B9" s="96" t="n">
         <x:f>COUNTIF('Checklist UAT'!F5:F142,"Cần DNH chốt công thức")+COUNTIF('Checklist UAT'!F5:F142,"Thiếu một phần dữ liệu")</x:f>
-        <x:v>65</x:v>
+        <x:v>62</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -1128,15 +1128,15 @@
         <x:v>S01</x:v>
       </x:c>
       <x:c r="F5" s="87" t="str">
-        <x:v>Thiếu một phần dữ liệu</x:v>
+        <x:v>Đủ nguồn</x:v>
       </x:c>
       <x:c r="G5" s="77" t="str">
-        <x:v>Kiểm phần có dữ liệu; phần thiếu phải được thông báo rõ</x:v>
+        <x:v>Đối chiếu số liệu, diễn giải và phân quyền</x:v>
       </x:c>
       <x:c r="H5" s="80" t="str"/>
       <x:c r="I5" s="81"/>
       <x:c r="J5" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K5" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu C01, checker S01.</x:v>
@@ -1193,7 +1193,7 @@
       <x:c r="H6" s="80" t="str"/>
       <x:c r="I6" s="81"/>
       <x:c r="J6" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K6" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu C02, checker S02.</x:v>
@@ -1250,7 +1250,7 @@
       <x:c r="H7" s="80" t="str"/>
       <x:c r="I7" s="81"/>
       <x:c r="J7" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K7" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu C03, checker S79.</x:v>
@@ -1307,7 +1307,7 @@
       <x:c r="H8" s="80" t="str"/>
       <x:c r="I8" s="81"/>
       <x:c r="J8" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K8" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu C04, checker S03.</x:v>
@@ -1364,7 +1364,7 @@
       <x:c r="H9" s="80" t="str"/>
       <x:c r="I9" s="81"/>
       <x:c r="J9" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K9" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu C05, checker S04.</x:v>
@@ -1421,7 +1421,7 @@
       <x:c r="H10" s="80" t="str"/>
       <x:c r="I10" s="81"/>
       <x:c r="J10" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K10" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu C06, checker S05.</x:v>
@@ -1478,7 +1478,7 @@
       <x:c r="H11" s="80" t="str"/>
       <x:c r="I11" s="81"/>
       <x:c r="J11" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K11" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu C07, checker S06.</x:v>
@@ -1535,7 +1535,7 @@
       <x:c r="H12" s="80" t="str"/>
       <x:c r="I12" s="81"/>
       <x:c r="J12" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K12" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu C08, checker S80.</x:v>
@@ -1592,7 +1592,7 @@
       <x:c r="H13" s="80" t="str"/>
       <x:c r="I13" s="81"/>
       <x:c r="J13" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K13" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu C09, checker S07.</x:v>
@@ -1649,7 +1649,7 @@
       <x:c r="H14" s="80" t="str"/>
       <x:c r="I14" s="81"/>
       <x:c r="J14" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K14" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu C10, checker S08.</x:v>
@@ -1706,7 +1706,7 @@
       <x:c r="H15" s="80" t="str"/>
       <x:c r="I15" s="81"/>
       <x:c r="J15" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K15" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu C11, checker S70.</x:v>
@@ -1763,7 +1763,7 @@
       <x:c r="H16" s="80" t="str"/>
       <x:c r="I16" s="81"/>
       <x:c r="J16" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K16" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu C12, checker S09.</x:v>
@@ -1820,7 +1820,7 @@
       <x:c r="H17" s="80" t="str"/>
       <x:c r="I17" s="81"/>
       <x:c r="J17" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K17" s="80" t="str">
         <x:v>Chatbot phải báo rõ chưa đủ dữ liệu/lịch sử; không tự tạo số.</x:v>
@@ -1877,7 +1877,7 @@
       <x:c r="H18" s="80" t="str"/>
       <x:c r="I18" s="81"/>
       <x:c r="J18" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K18" s="80" t="str">
         <x:v>Chatbot phải báo rõ chưa đủ dữ liệu/lịch sử; không tự tạo số.</x:v>
@@ -1934,7 +1934,7 @@
       <x:c r="H19" s="80" t="str"/>
       <x:c r="I19" s="81"/>
       <x:c r="J19" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K19" s="80" t="str">
         <x:v>Chatbot phải báo rõ chưa đủ dữ liệu/lịch sử; không tự tạo số.</x:v>
@@ -1991,7 +1991,7 @@
       <x:c r="H20" s="80" t="str"/>
       <x:c r="I20" s="81"/>
       <x:c r="J20" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K20" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu C16, checker S11.</x:v>
@@ -2048,7 +2048,7 @@
       <x:c r="H21" s="80" t="str"/>
       <x:c r="I21" s="81"/>
       <x:c r="J21" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K21" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu C17, checker S77.</x:v>
@@ -2105,7 +2105,7 @@
       <x:c r="H22" s="80" t="str"/>
       <x:c r="I22" s="81"/>
       <x:c r="J22" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K22" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu C18, checker S12.</x:v>
@@ -2162,7 +2162,7 @@
       <x:c r="H23" s="80" t="str"/>
       <x:c r="I23" s="81"/>
       <x:c r="J23" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K23" s="80" t="str">
         <x:v>Chatbot phải báo rõ chưa đủ dữ liệu/lịch sử; không tự tạo số.</x:v>
@@ -2219,7 +2219,7 @@
       <x:c r="H24" s="80" t="str"/>
       <x:c r="I24" s="81"/>
       <x:c r="J24" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K24" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu C20, checker S13.</x:v>
@@ -2276,7 +2276,7 @@
       <x:c r="H25" s="80" t="str"/>
       <x:c r="I25" s="81"/>
       <x:c r="J25" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K25" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu C21, checker S14.</x:v>
@@ -2333,7 +2333,7 @@
       <x:c r="H26" s="80" t="str"/>
       <x:c r="I26" s="81"/>
       <x:c r="J26" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K26" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu C22, checker S49.</x:v>
@@ -2390,7 +2390,7 @@
       <x:c r="H27" s="80" t="str"/>
       <x:c r="I27" s="81"/>
       <x:c r="J27" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K27" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu C23, checker S50.</x:v>
@@ -2447,7 +2447,7 @@
       <x:c r="H28" s="80" t="str"/>
       <x:c r="I28" s="81"/>
       <x:c r="J28" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K28" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu C24, checker S51.</x:v>
@@ -2504,7 +2504,7 @@
       <x:c r="H29" s="80" t="str"/>
       <x:c r="I29" s="81"/>
       <x:c r="J29" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K29" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu C25, checker S15.</x:v>
@@ -2561,7 +2561,7 @@
       <x:c r="H30" s="80" t="str"/>
       <x:c r="I30" s="81"/>
       <x:c r="J30" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K30" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu C26, checker S16.</x:v>
@@ -2618,7 +2618,7 @@
       <x:c r="H31" s="80" t="str"/>
       <x:c r="I31" s="81"/>
       <x:c r="J31" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K31" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu C27, checker S17.</x:v>
@@ -2675,7 +2675,7 @@
       <x:c r="H32" s="80" t="str"/>
       <x:c r="I32" s="81"/>
       <x:c r="J32" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K32" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu C28, checker S17.</x:v>
@@ -2732,7 +2732,7 @@
       <x:c r="H33" s="80" t="str"/>
       <x:c r="I33" s="81"/>
       <x:c r="J33" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K33" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu C29, checker S18.</x:v>
@@ -2789,7 +2789,7 @@
       <x:c r="H34" s="80" t="str"/>
       <x:c r="I34" s="81"/>
       <x:c r="J34" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K34" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu C30, checker S19.</x:v>
@@ -2846,7 +2846,7 @@
       <x:c r="H35" s="80" t="str"/>
       <x:c r="I35" s="81"/>
       <x:c r="J35" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K35" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu C31, checker S20.</x:v>
@@ -2903,7 +2903,7 @@
       <x:c r="H36" s="80" t="str"/>
       <x:c r="I36" s="81"/>
       <x:c r="J36" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K36" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu C32, checker S71.</x:v>
@@ -2960,7 +2960,7 @@
       <x:c r="H37" s="80" t="str"/>
       <x:c r="I37" s="81"/>
       <x:c r="J37" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K37" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu C33, checker S21.</x:v>
@@ -3017,7 +3017,7 @@
       <x:c r="H38" s="80" t="str"/>
       <x:c r="I38" s="81"/>
       <x:c r="J38" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K38" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu C34, checker S22.</x:v>
@@ -3074,7 +3074,7 @@
       <x:c r="H39" s="80" t="str"/>
       <x:c r="I39" s="81"/>
       <x:c r="J39" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K39" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu C35, checker S23.</x:v>
@@ -3131,7 +3131,7 @@
       <x:c r="H40" s="80" t="str"/>
       <x:c r="I40" s="81"/>
       <x:c r="J40" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K40" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu C36, checker S73.</x:v>
@@ -3188,7 +3188,7 @@
       <x:c r="H41" s="80" t="str"/>
       <x:c r="I41" s="81"/>
       <x:c r="J41" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K41" s="80" t="str">
         <x:v>Chatbot phải báo rõ chưa đủ dữ liệu/lịch sử; không tự tạo số.</x:v>
@@ -3245,7 +3245,7 @@
       <x:c r="H42" s="80" t="str"/>
       <x:c r="I42" s="81"/>
       <x:c r="J42" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K42" s="80" t="str">
         <x:v>Chatbot phải báo rõ chưa đủ dữ liệu/lịch sử; không tự tạo số.</x:v>
@@ -3302,7 +3302,7 @@
       <x:c r="H43" s="80" t="str"/>
       <x:c r="I43" s="81"/>
       <x:c r="J43" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K43" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu C39, checker S26.</x:v>
@@ -3359,7 +3359,7 @@
       <x:c r="H44" s="80" t="str"/>
       <x:c r="I44" s="81"/>
       <x:c r="J44" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K44" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu C40, checker S24.</x:v>
@@ -3405,21 +3405,21 @@
         <x:v>Giá trị tồn kho, số tháng tồn, hàng chậm luân chuyển, stock-out và hàng cận date thay đổi thế nào theo tháng?</x:v>
       </x:c>
       <x:c r="E45" s="87" t="str">
-        <x:v>S28</x:v>
+        <x:v>S27</x:v>
       </x:c>
       <x:c r="F45" s="87" t="str">
-        <x:v>Thiếu một phần dữ liệu</x:v>
+        <x:v>Chỉ có số hiện tại</x:v>
       </x:c>
       <x:c r="G45" s="77" t="str">
-        <x:v>Kiểm phần có dữ liệu; phần thiếu phải được thông báo rõ</x:v>
+        <x:v>Chỉ đối chiếu snapshot hiện tại</x:v>
       </x:c>
       <x:c r="H45" s="80" t="str"/>
       <x:c r="I45" s="81"/>
       <x:c r="J45" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K45" s="80" t="str">
-        <x:v>Đối chiếu file kết quả theo câu C41, checker S28.</x:v>
+        <x:v>Đối chiếu file kết quả theo câu C41, checker S27.</x:v>
       </x:c>
       <x:c r="L45" s="80" t="str"/>
       <x:c r="M45" s="88" t="str">
@@ -3473,7 +3473,7 @@
       <x:c r="H46" s="80" t="str"/>
       <x:c r="I46" s="81"/>
       <x:c r="J46" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K46" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu C42, checker S47.</x:v>
@@ -3530,7 +3530,7 @@
       <x:c r="H47" s="80" t="str"/>
       <x:c r="I47" s="81"/>
       <x:c r="J47" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K47" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu C43, checker S29.</x:v>
@@ -3587,7 +3587,7 @@
       <x:c r="H48" s="80" t="str"/>
       <x:c r="I48" s="81"/>
       <x:c r="J48" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K48" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu C44, checker S86.</x:v>
@@ -3633,7 +3633,7 @@
         <x:v>Tỷ lệ nhân sự đạt 65/70%, 80%, 100% và 120% KPI từng tháng theo kênh/miền/chức danh là bao nhiêu?</x:v>
       </x:c>
       <x:c r="E49" s="87" t="str">
-        <x:v>S31</x:v>
+        <x:v>S30</x:v>
       </x:c>
       <x:c r="F49" s="87" t="str">
         <x:v>Đủ nguồn</x:v>
@@ -3644,10 +3644,10 @@
       <x:c r="H49" s="80" t="str"/>
       <x:c r="I49" s="81"/>
       <x:c r="J49" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K49" s="80" t="str">
-        <x:v>Đối chiếu file kết quả theo câu C45, checker S31.</x:v>
+        <x:v>Đối chiếu file kết quả theo câu C45, checker S30.</x:v>
       </x:c>
       <x:c r="L49" s="80" t="str"/>
       <x:c r="M49" s="88" t="str">
@@ -3701,7 +3701,7 @@
       <x:c r="H50" s="80" t="str"/>
       <x:c r="I50" s="81"/>
       <x:c r="J50" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K50" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu C46, checker S32.</x:v>
@@ -3758,7 +3758,7 @@
       <x:c r="H51" s="80" t="str"/>
       <x:c r="I51" s="81"/>
       <x:c r="J51" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K51" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu C47, checker S64.</x:v>
@@ -3815,7 +3815,7 @@
       <x:c r="H52" s="80" t="str"/>
       <x:c r="I52" s="81"/>
       <x:c r="J52" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K52" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu C48, checker S33.</x:v>
@@ -3872,7 +3872,7 @@
       <x:c r="H53" s="80" t="str"/>
       <x:c r="I53" s="81"/>
       <x:c r="J53" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K53" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu C49, checker S34.</x:v>
@@ -3929,7 +3929,7 @@
       <x:c r="H54" s="80" t="str"/>
       <x:c r="I54" s="81"/>
       <x:c r="J54" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K54" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu C50, checker S35.</x:v>
@@ -3986,7 +3986,7 @@
       <x:c r="H55" s="80" t="str"/>
       <x:c r="I55" s="81"/>
       <x:c r="J55" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K55" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu C51, checker S82.</x:v>
@@ -4043,7 +4043,7 @@
       <x:c r="H56" s="80" t="str"/>
       <x:c r="I56" s="81"/>
       <x:c r="J56" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K56" s="80" t="str">
         <x:v>Chatbot phải báo rõ chưa đủ dữ liệu/lịch sử; không tự tạo số.</x:v>
@@ -4100,7 +4100,7 @@
       <x:c r="H57" s="80" t="str"/>
       <x:c r="I57" s="81"/>
       <x:c r="J57" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K57" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu C53, checker S37.</x:v>
@@ -4157,7 +4157,7 @@
       <x:c r="H58" s="80" t="str"/>
       <x:c r="I58" s="81"/>
       <x:c r="J58" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K58" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu C54, checker S38.</x:v>
@@ -4206,15 +4206,15 @@
         <x:v>S01</x:v>
       </x:c>
       <x:c r="F59" s="87" t="str">
-        <x:v>Thiếu một phần dữ liệu</x:v>
+        <x:v>Đủ nguồn</x:v>
       </x:c>
       <x:c r="G59" s="77" t="str">
-        <x:v>Kiểm phần có dữ liệu; phần thiếu phải được thông báo rõ</x:v>
+        <x:v>Đối chiếu số liệu, diễn giải và phân quyền</x:v>
       </x:c>
       <x:c r="H59" s="80" t="str"/>
       <x:c r="I59" s="81"/>
       <x:c r="J59" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K59" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu M01, checker S01.</x:v>
@@ -4271,7 +4271,7 @@
       <x:c r="H60" s="80" t="str"/>
       <x:c r="I60" s="81"/>
       <x:c r="J60" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K60" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu M02, checker S43.</x:v>
@@ -4328,7 +4328,7 @@
       <x:c r="H61" s="80" t="str"/>
       <x:c r="I61" s="81"/>
       <x:c r="J61" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K61" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu M03, checker S04.</x:v>
@@ -4385,7 +4385,7 @@
       <x:c r="H62" s="80" t="str"/>
       <x:c r="I62" s="81"/>
       <x:c r="J62" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K62" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu M04, checker S14.</x:v>
@@ -4442,7 +4442,7 @@
       <x:c r="H63" s="80" t="str"/>
       <x:c r="I63" s="81"/>
       <x:c r="J63" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K63" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu M05, checker S58.</x:v>
@@ -4499,7 +4499,7 @@
       <x:c r="H64" s="80" t="str"/>
       <x:c r="I64" s="81"/>
       <x:c r="J64" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K64" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu M06, checker S03.</x:v>
@@ -4556,7 +4556,7 @@
       <x:c r="H65" s="80" t="str"/>
       <x:c r="I65" s="81"/>
       <x:c r="J65" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K65" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu M07, checker S07.</x:v>
@@ -4613,7 +4613,7 @@
       <x:c r="H66" s="80" t="str"/>
       <x:c r="I66" s="81"/>
       <x:c r="J66" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K66" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu M08, checker S18.</x:v>
@@ -4670,7 +4670,7 @@
       <x:c r="H67" s="80" t="str"/>
       <x:c r="I67" s="81"/>
       <x:c r="J67" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K67" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu M09, checker S09.</x:v>
@@ -4727,7 +4727,7 @@
       <x:c r="H68" s="80" t="str"/>
       <x:c r="I68" s="81"/>
       <x:c r="J68" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K68" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu M10, checker S52.</x:v>
@@ -4784,7 +4784,7 @@
       <x:c r="H69" s="80" t="str"/>
       <x:c r="I69" s="81"/>
       <x:c r="J69" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K69" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu M11, checker S39.</x:v>
@@ -4841,7 +4841,7 @@
       <x:c r="H70" s="80" t="str"/>
       <x:c r="I70" s="81"/>
       <x:c r="J70" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K70" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu M12, checker S31.</x:v>
@@ -4898,7 +4898,7 @@
       <x:c r="H71" s="80" t="str"/>
       <x:c r="I71" s="81"/>
       <x:c r="J71" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K71" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu M13, checker S65.</x:v>
@@ -4955,7 +4955,7 @@
       <x:c r="H72" s="80" t="str"/>
       <x:c r="I72" s="81"/>
       <x:c r="J72" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K72" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu M14, checker S54.</x:v>
@@ -5012,7 +5012,7 @@
       <x:c r="H73" s="80" t="str"/>
       <x:c r="I73" s="81"/>
       <x:c r="J73" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K73" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu M15, checker S32.</x:v>
@@ -5069,7 +5069,7 @@
       <x:c r="H74" s="80" t="str"/>
       <x:c r="I74" s="81"/>
       <x:c r="J74" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K74" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu M16, checker S55.</x:v>
@@ -5126,7 +5126,7 @@
       <x:c r="H75" s="80" t="str"/>
       <x:c r="I75" s="81"/>
       <x:c r="J75" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K75" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu M17, checker S85.</x:v>
@@ -5183,7 +5183,7 @@
       <x:c r="H76" s="80" t="str"/>
       <x:c r="I76" s="81"/>
       <x:c r="J76" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K76" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu M18, checker S81.</x:v>
@@ -5240,7 +5240,7 @@
       <x:c r="H77" s="80" t="str"/>
       <x:c r="I77" s="81"/>
       <x:c r="J77" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K77" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu M19, checker S66.</x:v>
@@ -5297,7 +5297,7 @@
       <x:c r="H78" s="80" t="str"/>
       <x:c r="I78" s="81"/>
       <x:c r="J78" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K78" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu M20, checker S33.</x:v>
@@ -5354,7 +5354,7 @@
       <x:c r="H79" s="80" t="str"/>
       <x:c r="I79" s="81"/>
       <x:c r="J79" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K79" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu M21, checker S20.</x:v>
@@ -5411,7 +5411,7 @@
       <x:c r="H80" s="80" t="str"/>
       <x:c r="I80" s="81"/>
       <x:c r="J80" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K80" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu M22, checker S40.</x:v>
@@ -5468,7 +5468,7 @@
       <x:c r="H81" s="80" t="str"/>
       <x:c r="I81" s="81"/>
       <x:c r="J81" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K81" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu M23, checker S67.</x:v>
@@ -5525,7 +5525,7 @@
       <x:c r="H82" s="80" t="str"/>
       <x:c r="I82" s="81"/>
       <x:c r="J82" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K82" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu M24, checker S19.</x:v>
@@ -5582,7 +5582,7 @@
       <x:c r="H83" s="80" t="str"/>
       <x:c r="I83" s="81"/>
       <x:c r="J83" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K83" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu M25, checker S41.</x:v>
@@ -5639,7 +5639,7 @@
       <x:c r="H84" s="80" t="str"/>
       <x:c r="I84" s="81"/>
       <x:c r="J84" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K84" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu M26, checker S23.</x:v>
@@ -5696,7 +5696,7 @@
       <x:c r="H85" s="80" t="str"/>
       <x:c r="I85" s="81"/>
       <x:c r="J85" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K85" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu M27, checker S53.</x:v>
@@ -5753,7 +5753,7 @@
       <x:c r="H86" s="80" t="str"/>
       <x:c r="I86" s="81"/>
       <x:c r="J86" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K86" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu M28, checker S38.</x:v>
@@ -5810,7 +5810,7 @@
       <x:c r="H87" s="80" t="str"/>
       <x:c r="I87" s="81"/>
       <x:c r="J87" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K87" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu M29, checker S15.</x:v>
@@ -5867,7 +5867,7 @@
       <x:c r="H88" s="80" t="str"/>
       <x:c r="I88" s="81"/>
       <x:c r="J88" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K88" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu M30, checker S48.</x:v>
@@ -5924,7 +5924,7 @@
       <x:c r="H89" s="80" t="str"/>
       <x:c r="I89" s="81"/>
       <x:c r="J89" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K89" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu M31, checker S21.</x:v>
@@ -5981,7 +5981,7 @@
       <x:c r="H90" s="80" t="str"/>
       <x:c r="I90" s="81"/>
       <x:c r="J90" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K90" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu M32, checker S46.</x:v>
@@ -6038,7 +6038,7 @@
       <x:c r="H91" s="80" t="str"/>
       <x:c r="I91" s="81"/>
       <x:c r="J91" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K91" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu M33, checker S72.</x:v>
@@ -6095,7 +6095,7 @@
       <x:c r="H92" s="80" t="str"/>
       <x:c r="I92" s="81"/>
       <x:c r="J92" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K92" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu M34, checker S22.</x:v>
@@ -6152,7 +6152,7 @@
       <x:c r="H93" s="80" t="str"/>
       <x:c r="I93" s="81"/>
       <x:c r="J93" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K93" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu M35, checker S12.</x:v>
@@ -6209,7 +6209,7 @@
       <x:c r="H94" s="80" t="str"/>
       <x:c r="I94" s="81"/>
       <x:c r="J94" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K94" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu M36, checker S78.</x:v>
@@ -6266,7 +6266,7 @@
       <x:c r="H95" s="80" t="str"/>
       <x:c r="I95" s="81"/>
       <x:c r="J95" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K95" s="80" t="str">
         <x:v>Chatbot phải báo rõ chưa đủ dữ liệu/lịch sử; không tự tạo số.</x:v>
@@ -6323,7 +6323,7 @@
       <x:c r="H96" s="80" t="str"/>
       <x:c r="I96" s="81"/>
       <x:c r="J96" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K96" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu M38, checker S26.</x:v>
@@ -6380,7 +6380,7 @@
       <x:c r="H97" s="80" t="str"/>
       <x:c r="I97" s="81"/>
       <x:c r="J97" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K97" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu M39, checker S47.</x:v>
@@ -6437,7 +6437,7 @@
       <x:c r="H98" s="80" t="str"/>
       <x:c r="I98" s="81"/>
       <x:c r="J98" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K98" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu M40, checker S28.</x:v>
@@ -6494,7 +6494,7 @@
       <x:c r="H99" s="80" t="str"/>
       <x:c r="I99" s="81"/>
       <x:c r="J99" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K99" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu M41, checker S29.</x:v>
@@ -6551,7 +6551,7 @@
       <x:c r="H100" s="80" t="str"/>
       <x:c r="I100" s="81"/>
       <x:c r="J100" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K100" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu M42, checker S86.</x:v>
@@ -6608,7 +6608,7 @@
       <x:c r="H101" s="80" t="str"/>
       <x:c r="I101" s="81"/>
       <x:c r="J101" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K101" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu M43, checker S35.</x:v>
@@ -6665,7 +6665,7 @@
       <x:c r="H102" s="80" t="str"/>
       <x:c r="I102" s="81"/>
       <x:c r="J102" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K102" s="80" t="str">
         <x:v>Chatbot phải báo rõ chưa đủ dữ liệu/lịch sử; không tự tạo số.</x:v>
@@ -6722,7 +6722,7 @@
       <x:c r="H103" s="80" t="str"/>
       <x:c r="I103" s="81"/>
       <x:c r="J103" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K103" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu V01, checker S43.</x:v>
@@ -6779,7 +6779,7 @@
       <x:c r="H104" s="80" t="str"/>
       <x:c r="I104" s="81"/>
       <x:c r="J104" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K104" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu V02, checker S59.</x:v>
@@ -6836,7 +6836,7 @@
       <x:c r="H105" s="80" t="str"/>
       <x:c r="I105" s="81"/>
       <x:c r="J105" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K105" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu V03, checker S03.</x:v>
@@ -6893,7 +6893,7 @@
       <x:c r="H106" s="80" t="str"/>
       <x:c r="I106" s="81"/>
       <x:c r="J106" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K106" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu V04, checker S39.</x:v>
@@ -6950,7 +6950,7 @@
       <x:c r="H107" s="80" t="str"/>
       <x:c r="I107" s="81"/>
       <x:c r="J107" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K107" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu V05, checker S09.</x:v>
@@ -7007,7 +7007,7 @@
       <x:c r="H108" s="80" t="str"/>
       <x:c r="I108" s="81"/>
       <x:c r="J108" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K108" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu V06, checker S07.</x:v>
@@ -7064,7 +7064,7 @@
       <x:c r="H109" s="80" t="str"/>
       <x:c r="I109" s="81"/>
       <x:c r="J109" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K109" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu V07, checker S05.</x:v>
@@ -7121,7 +7121,7 @@
       <x:c r="H110" s="80" t="str"/>
       <x:c r="I110" s="81"/>
       <x:c r="J110" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K110" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu V08, checker S60.</x:v>
@@ -7178,7 +7178,7 @@
       <x:c r="H111" s="80" t="str"/>
       <x:c r="I111" s="81"/>
       <x:c r="J111" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K111" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu V09, checker S35.</x:v>
@@ -7235,7 +7235,7 @@
       <x:c r="H112" s="80" t="str"/>
       <x:c r="I112" s="81"/>
       <x:c r="J112" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K112" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu V10, checker S84.</x:v>
@@ -7292,7 +7292,7 @@
       <x:c r="H113" s="80" t="str"/>
       <x:c r="I113" s="81"/>
       <x:c r="J113" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K113" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu V11, checker S56.</x:v>
@@ -7349,7 +7349,7 @@
       <x:c r="H114" s="80" t="str"/>
       <x:c r="I114" s="81"/>
       <x:c r="J114" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K114" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu V12, checker S31.</x:v>
@@ -7406,7 +7406,7 @@
       <x:c r="H115" s="80" t="str"/>
       <x:c r="I115" s="81"/>
       <x:c r="J115" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K115" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu V13, checker S57.</x:v>
@@ -7463,7 +7463,7 @@
       <x:c r="H116" s="80" t="str"/>
       <x:c r="I116" s="81"/>
       <x:c r="J116" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K116" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu V14, checker S44.</x:v>
@@ -7520,7 +7520,7 @@
       <x:c r="H117" s="80" t="str"/>
       <x:c r="I117" s="81"/>
       <x:c r="J117" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K117" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu V15, checker S61.</x:v>
@@ -7577,7 +7577,7 @@
       <x:c r="H118" s="80" t="str"/>
       <x:c r="I118" s="81"/>
       <x:c r="J118" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K118" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu V16, checker S34.</x:v>
@@ -7634,7 +7634,7 @@
       <x:c r="H119" s="80" t="str"/>
       <x:c r="I119" s="81"/>
       <x:c r="J119" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K119" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu V17, checker S38.</x:v>
@@ -7691,7 +7691,7 @@
       <x:c r="H120" s="80" t="str"/>
       <x:c r="I120" s="81"/>
       <x:c r="J120" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K120" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu V18, checker S33.</x:v>
@@ -7748,7 +7748,7 @@
       <x:c r="H121" s="80" t="str"/>
       <x:c r="I121" s="81"/>
       <x:c r="J121" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K121" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu V19, checker S20.</x:v>
@@ -7805,7 +7805,7 @@
       <x:c r="H122" s="80" t="str"/>
       <x:c r="I122" s="81"/>
       <x:c r="J122" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K122" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu V20, checker S40.</x:v>
@@ -7862,7 +7862,7 @@
       <x:c r="H123" s="80" t="str"/>
       <x:c r="I123" s="81"/>
       <x:c r="J123" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K123" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu V21, checker S69.</x:v>
@@ -7919,7 +7919,7 @@
       <x:c r="H124" s="80" t="str"/>
       <x:c r="I124" s="81"/>
       <x:c r="J124" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K124" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu V22, checker S18.</x:v>
@@ -7976,7 +7976,7 @@
       <x:c r="H125" s="80" t="str"/>
       <x:c r="I125" s="81"/>
       <x:c r="J125" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K125" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu V23, checker S68.</x:v>
@@ -8033,7 +8033,7 @@
       <x:c r="H126" s="80" t="str"/>
       <x:c r="I126" s="81"/>
       <x:c r="J126" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K126" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu V24, checker S62.</x:v>
@@ -8090,7 +8090,7 @@
       <x:c r="H127" s="80" t="str"/>
       <x:c r="I127" s="81"/>
       <x:c r="J127" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K127" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu V25, checker S41.</x:v>
@@ -8147,7 +8147,7 @@
       <x:c r="H128" s="80" t="str"/>
       <x:c r="I128" s="81"/>
       <x:c r="J128" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K128" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu V26, checker S63.</x:v>
@@ -8204,7 +8204,7 @@
       <x:c r="H129" s="80" t="str"/>
       <x:c r="I129" s="81"/>
       <x:c r="J129" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K129" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu V27, checker S75.</x:v>
@@ -8261,7 +8261,7 @@
       <x:c r="H130" s="80" t="str"/>
       <x:c r="I130" s="81"/>
       <x:c r="J130" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K130" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu V28, checker S83.</x:v>
@@ -8318,7 +8318,7 @@
       <x:c r="H131" s="80" t="str"/>
       <x:c r="I131" s="81"/>
       <x:c r="J131" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K131" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu V29, checker S21.</x:v>
@@ -8375,7 +8375,7 @@
       <x:c r="H132" s="80" t="str"/>
       <x:c r="I132" s="81"/>
       <x:c r="J132" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K132" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu V30, checker S46.</x:v>
@@ -8432,7 +8432,7 @@
       <x:c r="H133" s="80" t="str"/>
       <x:c r="I133" s="81"/>
       <x:c r="J133" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K133" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu V31, checker S23.</x:v>
@@ -8489,7 +8489,7 @@
       <x:c r="H134" s="80" t="str"/>
       <x:c r="I134" s="81"/>
       <x:c r="J134" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K134" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu V32, checker S74.</x:v>
@@ -8546,7 +8546,7 @@
       <x:c r="H135" s="80" t="str"/>
       <x:c r="I135" s="81"/>
       <x:c r="J135" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K135" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu V33, checker S42.</x:v>
@@ -8603,7 +8603,7 @@
       <x:c r="H136" s="80" t="str"/>
       <x:c r="I136" s="81"/>
       <x:c r="J136" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K136" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu V34, checker S12.</x:v>
@@ -8660,7 +8660,7 @@
       <x:c r="H137" s="80" t="str"/>
       <x:c r="I137" s="81"/>
       <x:c r="J137" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K137" s="80" t="str">
         <x:v>Chatbot phải báo rõ chưa đủ dữ liệu/lịch sử; không tự tạo số.</x:v>
@@ -8717,7 +8717,7 @@
       <x:c r="H138" s="80" t="str"/>
       <x:c r="I138" s="81"/>
       <x:c r="J138" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K138" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu V36, checker S26.</x:v>
@@ -8774,7 +8774,7 @@
       <x:c r="H139" s="80" t="str"/>
       <x:c r="I139" s="81"/>
       <x:c r="J139" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K139" s="80" t="str">
         <x:v>Chatbot phải báo rõ chưa đủ dữ liệu/lịch sử; không tự tạo số.</x:v>
@@ -8831,7 +8831,7 @@
       <x:c r="H140" s="80" t="str"/>
       <x:c r="I140" s="81"/>
       <x:c r="J140" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K140" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu V38, checker S47.</x:v>
@@ -8888,7 +8888,7 @@
       <x:c r="H141" s="80" t="str"/>
       <x:c r="I141" s="81"/>
       <x:c r="J141" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K141" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu V39, checker S28.</x:v>
@@ -8945,7 +8945,7 @@
       <x:c r="H142" s="80" t="str"/>
       <x:c r="I142" s="81"/>
       <x:c r="J142" s="82" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="K142" s="80" t="str">
         <x:v>Đối chiếu file kết quả theo câu V40, checker S76.</x:v>
@@ -9006,7 +9006,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbb50b79844fe44b7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R06c10cecdca14a4a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9042,7 +9042,7 @@
         <x:v>Ngày chốt dữ liệu</x:v>
       </x:c>
       <x:c r="B3" s="16" t="n">
-        <x:v>46262</x:v>
+        <x:v>46265</x:v>
       </x:c>
     </x:row>
     <x:row r="4">

</xml_diff>